<commit_message>
UI pass 6: unify student/health data, disability filters, PDF cleanup
- Student list & profile now read the same data set: nickname /
  disability / old-new fall back to healthData (sheet) so the list
  matches the health menu. nickname column backfilled + sheet import
  now stores it.
- ข้อมูลนักเรียน: two disability-type filters (1-7, supports students
  with two types), colored เด็กเก่า/ใหม่ chips, and the PDF export now
  uses the new columns.
- Health/medication menu PDF: export a curated set of key columns
  instead of dumping all ~33 sheet columns (was unreadable).
- Student form + Excel import + template gain ประเภทความพิการ,
  เด็กเก่า/ใหม่, เลขบัตรประชาชน, ที่อยู่, น้ำหนัก/ส่วนสูง, สิทธิ — stored
  into healthData so all views stay in sync.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/public/ksp_save_students_template.xlsx
+++ b/frontend/public/ksp_save_students_template.xlsx
@@ -397,23 +397,30 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:V2"/>
   <cols>
-    <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="1" max="1" width="15.83203125" customWidth="1"/>
+    <col min="2" max="2" width="17.83203125" customWidth="1"/>
     <col min="3" max="3" width="12.83203125" customWidth="1"/>
     <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="13.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
     <col min="7" max="7" width="16.83203125" customWidth="1"/>
-    <col min="8" max="8" width="21.83203125" customWidth="1"/>
-    <col min="9" max="9" width="14.83203125" customWidth="1"/>
+    <col min="8" max="8" width="12.83203125" customWidth="1"/>
+    <col min="9" max="9" width="12.83203125" customWidth="1"/>
     <col min="10" max="10" width="15.83203125" customWidth="1"/>
-    <col min="11" max="11" width="15.83203125" customWidth="1"/>
-    <col min="12" max="12" width="14.83203125" customWidth="1"/>
-    <col min="13" max="13" width="13.83203125" customWidth="1"/>
+    <col min="11" max="11" width="20.83203125" customWidth="1"/>
+    <col min="12" max="12" width="13.83203125" customWidth="1"/>
+    <col min="13" max="13" width="12.83203125" customWidth="1"/>
     <col min="14" max="14" width="12.83203125" customWidth="1"/>
     <col min="15" max="15" width="12.83203125" customWidth="1"/>
+    <col min="16" max="16" width="14.83203125" customWidth="1"/>
+    <col min="17" max="17" width="14.83203125" customWidth="1"/>
+    <col min="18" max="18" width="13.83203125" customWidth="1"/>
+    <col min="19" max="19" width="12.83203125" customWidth="1"/>
+    <col min="20" max="20" width="12.83203125" customWidth="1"/>
+    <col min="21" max="21" width="12.83203125" customWidth="1"/>
+    <col min="22" max="22" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -421,45 +428,66 @@
         <v>รหัสนักเรียน</v>
       </c>
       <c r="B1" t="str">
+        <v>เลขบัตรประชาชน</v>
+      </c>
+      <c r="C1" t="str">
         <v>ชื่อ</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>นามสกุล</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>ชื่อเล่น</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
+        <v>ประเภทความพิการ</v>
+      </c>
+      <c r="G1" t="str">
+        <v>เด็กเก่า/ใหม่</v>
+      </c>
+      <c r="H1" t="str">
         <v>ชั้นเรียน</v>
       </c>
-      <c r="F1" t="str">
+      <c r="I1" t="str">
         <v>เรือนนอน</v>
       </c>
-      <c r="G1" t="str">
+      <c r="J1" t="str">
         <v>ครูประจำชั้น</v>
       </c>
-      <c r="H1" t="str">
+      <c r="K1" t="str">
         <v>เบอร์ครูประจำชั้น</v>
       </c>
-      <c r="I1" t="str">
+      <c r="L1" t="str">
         <v>กรุ๊ปเลือด</v>
       </c>
-      <c r="J1" t="str">
+      <c r="M1" t="str">
+        <v>น้ำหนัก</v>
+      </c>
+      <c r="N1" t="str">
+        <v>ส่วนสูง</v>
+      </c>
+      <c r="O1" t="str">
+        <v>สิทธิ</v>
+      </c>
+      <c r="P1" t="str">
         <v>โรคประจำตัว</v>
       </c>
-      <c r="K1" t="str">
+      <c r="Q1" t="str">
         <v>แพ้ยา/อาหาร</v>
       </c>
-      <c r="L1" t="str">
+      <c r="R1" t="str">
         <v>ยาประจำตัว</v>
       </c>
-      <c r="M1" t="str">
+      <c r="S1" t="str">
         <v>ผู้ปกครอง</v>
       </c>
-      <c r="N1" t="str">
+      <c r="T1" t="str">
         <v>เบอร์โทร</v>
       </c>
-      <c r="O1" t="str">
+      <c r="U1" t="str">
+        <v>ที่อยู่</v>
+      </c>
+      <c r="V1" t="str">
         <v>สถานะ</v>
       </c>
     </row>
@@ -468,51 +496,72 @@
         <v>6601001</v>
       </c>
       <c r="B2" t="str">
+        <v>1234567890123</v>
+      </c>
+      <c r="C2" t="str">
         <v>สมชาย</v>
       </c>
-      <c r="C2" t="str">
+      <c r="D2" t="str">
         <v>ใจดี</v>
       </c>
-      <c r="D2" t="str">
+      <c r="E2" t="str">
         <v>ชาย</v>
       </c>
-      <c r="E2" t="str">
+      <c r="F2" t="str">
+        <v>7 (ออทิสติก)</v>
+      </c>
+      <c r="G2" t="str">
+        <v>ใหม่</v>
+      </c>
+      <c r="H2" t="str">
         <v>ป.1</v>
       </c>
-      <c r="F2" t="str">
+      <c r="I2" t="str">
         <v>แพรวา</v>
       </c>
-      <c r="G2" t="str">
+      <c r="J2" t="str">
         <v>ครูสมหญิง</v>
       </c>
-      <c r="H2" t="str">
+      <c r="K2" t="str">
         <v>081-0000000</v>
       </c>
-      <c r="I2" t="str">
+      <c r="L2" t="str">
         <v>O</v>
       </c>
-      <c r="J2" t="str">
+      <c r="M2" t="str">
+        <v>35</v>
+      </c>
+      <c r="N2" t="str">
+        <v>130</v>
+      </c>
+      <c r="O2" t="str">
+        <v>บัตรทอง</v>
+      </c>
+      <c r="P2" t="str">
         <v>-</v>
       </c>
-      <c r="K2" t="str">
+      <c r="Q2" t="str">
         <v>-</v>
       </c>
-      <c r="L2" t="str">
+      <c r="R2" t="str">
         <v>-</v>
       </c>
-      <c r="M2" t="str">
+      <c r="S2" t="str">
         <v>นางสมศรี ใจดี</v>
       </c>
-      <c r="N2" t="str">
+      <c r="T2" t="str">
         <v>089-0000000</v>
       </c>
-      <c r="O2" t="str">
+      <c r="U2" t="str">
+        <v>1 ม.1 ต.- อ.- จ.กาฬสินธุ์</v>
+      </c>
+      <c r="V2" t="str">
         <v>ประจำ</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 5 health-summary menus (disease/nutrition/physical/contraception/injection)
- New /health-reports/:type endpoint builds school-wide summaries from
  the existing student data, with measurement criteria and (nutrition)
  status counts. Generic HealthReportPage + 5 sidebar menus + routes.
- Reproductive-health fields (menstruation, contraception method/dates,
  injection date/place/next/side-effects) and physical-result /
  allergy-symptom added to healthData via the student form, Excel
  import + template, and shown in the detail view. Contraception &
  injection data imported from their Google Sheets by name match.
- PDF export default font is now 14pt.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/public/ksp_save_students_template.xlsx
+++ b/frontend/public/ksp_save_students_template.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V2"/>
+  <dimension ref="A1:AC2"/>
   <cols>
     <col min="1" max="1" width="15.83203125" customWidth="1"/>
     <col min="2" max="2" width="17.83203125" customWidth="1"/>
@@ -416,11 +416,18 @@
     <col min="15" max="15" width="12.83203125" customWidth="1"/>
     <col min="16" max="16" width="14.83203125" customWidth="1"/>
     <col min="17" max="17" width="14.83203125" customWidth="1"/>
-    <col min="18" max="18" width="13.83203125" customWidth="1"/>
-    <col min="19" max="19" width="12.83203125" customWidth="1"/>
-    <col min="20" max="20" width="12.83203125" customWidth="1"/>
+    <col min="18" max="18" width="18.83203125" customWidth="1"/>
+    <col min="19" max="19" width="16.83203125" customWidth="1"/>
+    <col min="20" max="20" width="13.83203125" customWidth="1"/>
     <col min="21" max="21" width="12.83203125" customWidth="1"/>
     <col min="22" max="22" width="12.83203125" customWidth="1"/>
+    <col min="23" max="23" width="12.83203125" customWidth="1"/>
+    <col min="24" max="24" width="18.83203125" customWidth="1"/>
+    <col min="25" max="25" width="15.83203125" customWidth="1"/>
+    <col min="26" max="26" width="23.83203125" customWidth="1"/>
+    <col min="27" max="27" width="18.83203125" customWidth="1"/>
+    <col min="28" max="28" width="24.83203125" customWidth="1"/>
+    <col min="29" max="29" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -476,18 +483,39 @@
         <v>แพ้ยา/อาหาร</v>
       </c>
       <c r="R1" t="str">
+        <v>อาการแสดงการแพ้</v>
+      </c>
+      <c r="S1" t="str">
+        <v>ผลตรวจร่างกาย</v>
+      </c>
+      <c r="T1" t="str">
         <v>ยาประจำตัว</v>
       </c>
-      <c r="S1" t="str">
+      <c r="U1" t="str">
         <v>ผู้ปกครอง</v>
       </c>
-      <c r="T1" t="str">
+      <c r="V1" t="str">
         <v>เบอร์โทร</v>
       </c>
-      <c r="U1" t="str">
+      <c r="W1" t="str">
         <v>ที่อยู่</v>
       </c>
-      <c r="V1" t="str">
+      <c r="X1" t="str">
+        <v>การมีประจำเดือน</v>
+      </c>
+      <c r="Y1" t="str">
+        <v>การคุมกำเนิด</v>
+      </c>
+      <c r="Z1" t="str">
+        <v>วันที่ฉีดยาคุมล่าสุด</v>
+      </c>
+      <c r="AA1" t="str">
+        <v>สถานที่ฉีดยาคุม</v>
+      </c>
+      <c r="AB1" t="str">
+        <v>นัดฉีดยาคุมครั้งถัดไป</v>
+      </c>
+      <c r="AC1" t="str">
         <v>สถานะ</v>
       </c>
     </row>
@@ -496,7 +524,7 @@
         <v>6601001</v>
       </c>
       <c r="B2" t="str">
-        <v>1234567890123</v>
+        <v/>
       </c>
       <c r="C2" t="str">
         <v>สมชาย</v>
@@ -508,10 +536,10 @@
         <v>ชาย</v>
       </c>
       <c r="F2" t="str">
-        <v>7 (ออทิสติก)</v>
+        <v/>
       </c>
       <c r="G2" t="str">
-        <v>ใหม่</v>
+        <v/>
       </c>
       <c r="H2" t="str">
         <v>ป.1</v>
@@ -520,48 +548,69 @@
         <v>แพรวา</v>
       </c>
       <c r="J2" t="str">
-        <v>ครูสมหญิง</v>
+        <v/>
       </c>
       <c r="K2" t="str">
-        <v>081-0000000</v>
+        <v/>
       </c>
       <c r="L2" t="str">
         <v>O</v>
       </c>
       <c r="M2" t="str">
-        <v>35</v>
+        <v/>
       </c>
       <c r="N2" t="str">
-        <v>130</v>
+        <v/>
       </c>
       <c r="O2" t="str">
-        <v>บัตรทอง</v>
+        <v/>
       </c>
       <c r="P2" t="str">
-        <v>-</v>
+        <v/>
       </c>
       <c r="Q2" t="str">
-        <v>-</v>
+        <v/>
       </c>
       <c r="R2" t="str">
-        <v>-</v>
+        <v/>
       </c>
       <c r="S2" t="str">
-        <v>นางสมศรี ใจดี</v>
+        <v/>
       </c>
       <c r="T2" t="str">
-        <v>089-0000000</v>
+        <v/>
       </c>
       <c r="U2" t="str">
-        <v>1 ม.1 ต.- อ.- จ.กาฬสินธุ์</v>
+        <v/>
       </c>
       <c r="V2" t="str">
+        <v/>
+      </c>
+      <c r="W2" t="str">
+        <v/>
+      </c>
+      <c r="X2" t="str">
+        <v/>
+      </c>
+      <c r="Y2" t="str">
+        <v/>
+      </c>
+      <c r="Z2" t="str">
+        <v/>
+      </c>
+      <c r="AA2" t="str">
+        <v/>
+      </c>
+      <c r="AB2" t="str">
+        <v/>
+      </c>
+      <c r="AC2" t="str">
         <v>ประจำ</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AC2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Birthdate picker, table-style profile, medication time columns, report polish
- Student form: วันเดือนปีเกิด via native date picker (iOS wheel),
  ISO<->Thai-BE conversion; added to Excel/CSV template + importer.
- Profile/detail: section headers are now centered blue table-header
  bars (white text); reproductive-health fields shown.
- Medication menu: รายการยา split into per-meal columns
  (เช้า/กลางวัน/เย็น each with ก่อน/หลังอาหาร, plus ก่อนนอน, นอกเวลา),
  one stacked sub-row per drug, driven by structured data from the API.
- Health reports: criteria moved below the table, summary chips moved
  in front of the search box, table raised; nutrition rows colored by
  status (สมส่วน=green/ผอม=yellow/ท้วม=orange/อ้วน=red/อื่นๆ=blue);
  injection rows turn orange when the next appointment is within 7 days.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/public/ksp_save_students_template.xlsx
+++ b/frontend/public/ksp_save_students_template.xlsx
@@ -397,37 +397,38 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AC2"/>
+  <dimension ref="A1:AD2"/>
   <cols>
     <col min="1" max="1" width="15.83203125" customWidth="1"/>
     <col min="2" max="2" width="17.83203125" customWidth="1"/>
     <col min="3" max="3" width="12.83203125" customWidth="1"/>
     <col min="4" max="4" width="12.83203125" customWidth="1"/>
     <col min="5" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="18.83203125" customWidth="1"/>
-    <col min="7" max="7" width="16.83203125" customWidth="1"/>
-    <col min="8" max="8" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="17.83203125" customWidth="1"/>
+    <col min="7" max="7" width="18.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
     <col min="9" max="9" width="12.83203125" customWidth="1"/>
-    <col min="10" max="10" width="15.83203125" customWidth="1"/>
-    <col min="11" max="11" width="20.83203125" customWidth="1"/>
-    <col min="12" max="12" width="13.83203125" customWidth="1"/>
-    <col min="13" max="13" width="12.83203125" customWidth="1"/>
+    <col min="10" max="10" width="12.83203125" customWidth="1"/>
+    <col min="11" max="11" width="15.83203125" customWidth="1"/>
+    <col min="12" max="12" width="20.83203125" customWidth="1"/>
+    <col min="13" max="13" width="13.83203125" customWidth="1"/>
     <col min="14" max="14" width="12.83203125" customWidth="1"/>
     <col min="15" max="15" width="12.83203125" customWidth="1"/>
-    <col min="16" max="16" width="14.83203125" customWidth="1"/>
+    <col min="16" max="16" width="12.83203125" customWidth="1"/>
     <col min="17" max="17" width="14.83203125" customWidth="1"/>
-    <col min="18" max="18" width="18.83203125" customWidth="1"/>
-    <col min="19" max="19" width="16.83203125" customWidth="1"/>
-    <col min="20" max="20" width="13.83203125" customWidth="1"/>
-    <col min="21" max="21" width="12.83203125" customWidth="1"/>
+    <col min="18" max="18" width="14.83203125" customWidth="1"/>
+    <col min="19" max="19" width="18.83203125" customWidth="1"/>
+    <col min="20" max="20" width="16.83203125" customWidth="1"/>
+    <col min="21" max="21" width="13.83203125" customWidth="1"/>
     <col min="22" max="22" width="12.83203125" customWidth="1"/>
     <col min="23" max="23" width="12.83203125" customWidth="1"/>
-    <col min="24" max="24" width="18.83203125" customWidth="1"/>
-    <col min="25" max="25" width="15.83203125" customWidth="1"/>
-    <col min="26" max="26" width="23.83203125" customWidth="1"/>
-    <col min="27" max="27" width="18.83203125" customWidth="1"/>
-    <col min="28" max="28" width="24.83203125" customWidth="1"/>
-    <col min="29" max="29" width="12.83203125" customWidth="1"/>
+    <col min="24" max="24" width="12.83203125" customWidth="1"/>
+    <col min="25" max="25" width="18.83203125" customWidth="1"/>
+    <col min="26" max="26" width="15.83203125" customWidth="1"/>
+    <col min="27" max="27" width="23.83203125" customWidth="1"/>
+    <col min="28" max="28" width="18.83203125" customWidth="1"/>
+    <col min="29" max="29" width="24.83203125" customWidth="1"/>
+    <col min="30" max="30" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -447,75 +448,78 @@
         <v>ชื่อเล่น</v>
       </c>
       <c r="F1" t="str">
+        <v>วันเดือนปีเกิด</v>
+      </c>
+      <c r="G1" t="str">
         <v>ประเภทความพิการ</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>เด็กเก่า/ใหม่</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>ชั้นเรียน</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>เรือนนอน</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>ครูประจำชั้น</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>เบอร์ครูประจำชั้น</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>กรุ๊ปเลือด</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>น้ำหนัก</v>
       </c>
-      <c r="N1" t="str">
+      <c r="O1" t="str">
         <v>ส่วนสูง</v>
       </c>
-      <c r="O1" t="str">
+      <c r="P1" t="str">
         <v>สิทธิ</v>
       </c>
-      <c r="P1" t="str">
+      <c r="Q1" t="str">
         <v>โรคประจำตัว</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="R1" t="str">
         <v>แพ้ยา/อาหาร</v>
       </c>
-      <c r="R1" t="str">
+      <c r="S1" t="str">
         <v>อาการแสดงการแพ้</v>
       </c>
-      <c r="S1" t="str">
+      <c r="T1" t="str">
         <v>ผลตรวจร่างกาย</v>
       </c>
-      <c r="T1" t="str">
+      <c r="U1" t="str">
         <v>ยาประจำตัว</v>
       </c>
-      <c r="U1" t="str">
+      <c r="V1" t="str">
         <v>ผู้ปกครอง</v>
       </c>
-      <c r="V1" t="str">
+      <c r="W1" t="str">
         <v>เบอร์โทร</v>
       </c>
-      <c r="W1" t="str">
+      <c r="X1" t="str">
         <v>ที่อยู่</v>
       </c>
-      <c r="X1" t="str">
+      <c r="Y1" t="str">
         <v>การมีประจำเดือน</v>
       </c>
-      <c r="Y1" t="str">
+      <c r="Z1" t="str">
         <v>การคุมกำเนิด</v>
       </c>
-      <c r="Z1" t="str">
+      <c r="AA1" t="str">
         <v>วันที่ฉีดยาคุมล่าสุด</v>
       </c>
-      <c r="AA1" t="str">
+      <c r="AB1" t="str">
         <v>สถานที่ฉีดยาคุม</v>
       </c>
-      <c r="AB1" t="str">
+      <c r="AC1" t="str">
         <v>นัดฉีดยาคุมครั้งถัดไป</v>
       </c>
-      <c r="AC1" t="str">
+      <c r="AD1" t="str">
         <v>สถานะ</v>
       </c>
     </row>
@@ -536,29 +540,29 @@
         <v>ชาย</v>
       </c>
       <c r="F2" t="str">
-        <v/>
+        <v>3/2/2556</v>
       </c>
       <c r="G2" t="str">
         <v/>
       </c>
       <c r="H2" t="str">
+        <v/>
+      </c>
+      <c r="I2" t="str">
         <v>ป.1</v>
       </c>
-      <c r="I2" t="str">
+      <c r="J2" t="str">
         <v>แพรวา</v>
       </c>
-      <c r="J2" t="str">
-        <v/>
-      </c>
       <c r="K2" t="str">
         <v/>
       </c>
       <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
         <v>O</v>
       </c>
-      <c r="M2" t="str">
-        <v/>
-      </c>
       <c r="N2" t="str">
         <v/>
       </c>
@@ -605,12 +609,15 @@
         <v/>
       </c>
       <c r="AC2" t="str">
+        <v/>
+      </c>
+      <c r="AD2" t="str">
         <v>ประจำ</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AC2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AD2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>